<commit_message>
fine tune asset modelling and refactor some code
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/resources/templates/LEV.xlsx
+++ b/epsilon-phi-core/src/resources/templates/LEV.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B60614CC-E7E9-864A-B653-20679F3ACEB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B21C1AD-B26B-F24E-9A35-15552081EEBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3580" yWindow="2500" windowWidth="27240" windowHeight="16440" xr2:uid="{248642D4-931A-B040-A0E6-CA770CD233B6}"/>
+    <workbookView xWindow="3580" yWindow="2500" windowWidth="27240" windowHeight="16440" activeTab="1" xr2:uid="{248642D4-931A-B040-A0E6-CA770CD233B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Lev" sheetId="1" r:id="rId1"/>
+    <sheet name="Lev2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="1">
   <si>
     <t>BDLEVG</t>
   </si>
@@ -2044,4 +2045,1543 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87888A2A-E60A-B44B-A5CE-99D0D2CBCCF8}">
+  <dimension ref="A1:B200"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>24926</v>
+      </c>
+      <c r="B2" s="2">
+        <v>-2.5612229009999998E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>25017</v>
+      </c>
+      <c r="B3" s="2">
+        <v>8.9705673100000001E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>25111</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.17297228220000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>25203</v>
+      </c>
+      <c r="B5" s="2">
+        <v>-0.11152793470000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>25293</v>
+      </c>
+      <c r="B6" s="2">
+        <v>-0.12521450149999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>25384</v>
+      </c>
+      <c r="B7" s="2">
+        <v>3.5691832229999998E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>25476</v>
+      </c>
+      <c r="B8" s="2">
+        <v>-6.8988612960000001E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>25568</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0.13479961260000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>25658</v>
+      </c>
+      <c r="B10" s="2">
+        <v>4.653465281E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>25749</v>
+      </c>
+      <c r="B11" s="2">
+        <v>-7.0820004699999994E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>25841</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0.21818404319999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>25933</v>
+      </c>
+      <c r="B13" s="2">
+        <v>7.8159675100000006E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>26023</v>
+      </c>
+      <c r="B14" s="2">
+        <v>2.0531746890000001E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>26114</v>
+      </c>
+      <c r="B15" s="2">
+        <v>-9.2944299150000007E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
+        <v>26206</v>
+      </c>
+      <c r="B16" s="2">
+        <v>9.5784780300000004E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>26298</v>
+      </c>
+      <c r="B17" s="2">
+        <v>6.7280107099999993E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="3">
+        <v>26389</v>
+      </c>
+      <c r="B18" s="2">
+        <v>-5.5053728499999998E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>26480</v>
+      </c>
+      <c r="B19" s="2">
+        <v>-1.3755574960000001E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>26571</v>
+      </c>
+      <c r="B20" s="2">
+        <v>5.2840279819999995E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>26662</v>
+      </c>
+      <c r="B21" s="2">
+        <v>4.1172256089999998E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <v>26753</v>
+      </c>
+      <c r="B22" s="2">
+        <v>-0.19987061549999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>26844</v>
+      </c>
+      <c r="B23" s="2">
+        <v>-0.14052204309999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>26935</v>
+      </c>
+      <c r="B24" s="2">
+        <v>-9.8271914070000008E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>27029</v>
+      </c>
+      <c r="B25" s="2">
+        <v>-5.4387755090000003E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>27117</v>
+      </c>
+      <c r="B26" s="2">
+        <v>-0.11701305209999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <v>27208</v>
+      </c>
+      <c r="B27" s="2">
+        <v>4.1188576100000002E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>27302</v>
+      </c>
+      <c r="B28" s="2">
+        <v>-1.0938205580000001E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>27394</v>
+      </c>
+      <c r="B29" s="2">
+        <v>-0.14443440439999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <v>27484</v>
+      </c>
+      <c r="B30" s="2">
+        <v>9.2312160259999998E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>27575</v>
+      </c>
+      <c r="B31" s="2">
+        <v>3.667034466E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>27667</v>
+      </c>
+      <c r="B32" s="2">
+        <v>-1.7008418810000002E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>27759</v>
+      </c>
+      <c r="B33" s="2">
+        <v>4.7062768899999996E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <v>27850</v>
+      </c>
+      <c r="B34" s="2">
+        <v>0.33283150849999998</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>27941</v>
+      </c>
+      <c r="B35" s="2">
+        <v>7.1559856850000006E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="3">
+        <v>28033</v>
+      </c>
+      <c r="B36" s="2">
+        <v>0.20154922630000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <v>28125</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1.5983291760000001E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>28215</v>
+      </c>
+      <c r="B38" s="2">
+        <v>1.7465102450000002E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>28306</v>
+      </c>
+      <c r="B39" s="2">
+        <v>8.6535824980000009E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <v>28398</v>
+      </c>
+      <c r="B40" s="2">
+        <v>4.1394794509999999E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="3">
+        <v>28489</v>
+      </c>
+      <c r="B41" s="2">
+        <v>-2.1195698570000001E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="3">
+        <v>28580</v>
+      </c>
+      <c r="B42" s="2">
+        <v>0.15482554130000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="3">
+        <v>28671</v>
+      </c>
+      <c r="B43" s="2">
+        <v>4.6685042489999995E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="3">
+        <v>28762</v>
+      </c>
+      <c r="B44" s="2">
+        <v>5.5049332480000004E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <v>28853</v>
+      </c>
+      <c r="B45" s="2">
+        <v>-9.5263042939999987E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>28944</v>
+      </c>
+      <c r="B46" s="2">
+        <v>8.9114690509999997E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>29035</v>
+      </c>
+      <c r="B47" s="2">
+        <v>0.20890656830000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>29126</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2.1828087109999998E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>29220</v>
+      </c>
+      <c r="B49" s="2">
+        <v>-0.1748676522</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <v>29311</v>
+      </c>
+      <c r="B50" s="2">
+        <v>4.9649324259999995E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" s="3">
+        <v>29402</v>
+      </c>
+      <c r="B51" s="2">
+        <v>1.6790601360000001E-2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>29494</v>
+      </c>
+      <c r="B52" s="2">
+        <v>1.5445800700000002E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="3">
+        <v>29586</v>
+      </c>
+      <c r="B53" s="2">
+        <v>-1.7741891039999999E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="3">
+        <v>29676</v>
+      </c>
+      <c r="B54" s="2">
+        <v>8.9443659629999991E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="3">
+        <v>29767</v>
+      </c>
+      <c r="B55" s="2">
+        <v>-1.971310636E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="3">
+        <v>29859</v>
+      </c>
+      <c r="B56" s="2">
+        <v>6.802147486E-2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="3">
+        <v>29951</v>
+      </c>
+      <c r="B57" s="2">
+        <v>7.5194304850000004E-2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="3">
+        <v>30041</v>
+      </c>
+      <c r="B58" s="2">
+        <v>-3.0849620940000003E-2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="3">
+        <v>30132</v>
+      </c>
+      <c r="B59" s="2">
+        <v>3.7887095099999997E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="3">
+        <v>30224</v>
+      </c>
+      <c r="B60" s="2">
+        <v>7.9774452780000005E-2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="3">
+        <v>30316</v>
+      </c>
+      <c r="B61" s="2">
+        <v>-7.9371802300000002E-2</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="3">
+        <v>30406</v>
+      </c>
+      <c r="B62" s="2">
+        <v>-1.429593294E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" s="3">
+        <v>30497</v>
+      </c>
+      <c r="B63" s="2">
+        <v>8.5411739600000005E-3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" s="3">
+        <v>30589</v>
+      </c>
+      <c r="B64" s="2">
+        <v>0.11251476789999999</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" s="3">
+        <v>30680</v>
+      </c>
+      <c r="B65" s="2">
+        <v>-2.0038088300000003E-3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" s="3">
+        <v>30771</v>
+      </c>
+      <c r="B66" s="2">
+        <v>6.1725001300000006E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" s="3">
+        <v>30862</v>
+      </c>
+      <c r="B67" s="2">
+        <v>4.091850591E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" s="3">
+        <v>30953</v>
+      </c>
+      <c r="B68" s="2">
+        <v>4.315360847E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" s="3">
+        <v>31047</v>
+      </c>
+      <c r="B69" s="2">
+        <v>8.0121620830000004E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="3">
+        <v>31135</v>
+      </c>
+      <c r="B70" s="2">
+        <v>-5.1824019239999998E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="3">
+        <v>31226</v>
+      </c>
+      <c r="B71" s="2">
+        <v>2.6878398159999997E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" s="3">
+        <v>31320</v>
+      </c>
+      <c r="B72" s="2">
+        <v>2.1666490409999999E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="3">
+        <v>31412</v>
+      </c>
+      <c r="B73" s="2">
+        <v>1.742013928E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="3">
+        <v>31502</v>
+      </c>
+      <c r="B74" s="2">
+        <v>5.541538276E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="3">
+        <v>31593</v>
+      </c>
+      <c r="B75" s="2">
+        <v>-2.2498889670000001E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="3">
+        <v>31685</v>
+      </c>
+      <c r="B76" s="2">
+        <v>3.26507043E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" s="3">
+        <v>31777</v>
+      </c>
+      <c r="B77" s="2">
+        <v>-7.4213376309999995E-2</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" s="3">
+        <v>31867</v>
+      </c>
+      <c r="B78" s="2">
+        <v>2.8265701970000001E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" s="3">
+        <v>31958</v>
+      </c>
+      <c r="B79" s="2">
+        <v>-8.765591369999999E-3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" s="3">
+        <v>32050</v>
+      </c>
+      <c r="B80" s="2">
+        <v>6.9589662309999994E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" s="3">
+        <v>32142</v>
+      </c>
+      <c r="B81" s="2">
+        <v>-9.3020262329999992E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" s="3">
+        <v>32233</v>
+      </c>
+      <c r="B82" s="2">
+        <v>0.10769419579999999</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" s="3">
+        <v>32324</v>
+      </c>
+      <c r="B83" s="2">
+        <v>-2.6214862289999998E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" s="3">
+        <v>32416</v>
+      </c>
+      <c r="B84" s="2">
+        <v>6.4366326670000001E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" s="3">
+        <v>32507</v>
+      </c>
+      <c r="B85" s="2">
+        <v>-0.10973022809999999</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" s="3">
+        <v>32598</v>
+      </c>
+      <c r="B86" s="2">
+        <v>0.18978207300000002</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" s="3">
+        <v>32689</v>
+      </c>
+      <c r="B87" s="2">
+        <v>0.12654858759999998</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" s="3">
+        <v>32780</v>
+      </c>
+      <c r="B88" s="2">
+        <v>-7.6282724070000002E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89" s="3">
+        <v>32871</v>
+      </c>
+      <c r="B89" s="2">
+        <v>-2.8852190310000001E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90" s="3">
+        <v>32962</v>
+      </c>
+      <c r="B90" s="2">
+        <v>7.9572753689999998E-2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91" s="3">
+        <v>33053</v>
+      </c>
+      <c r="B91" s="2">
+        <v>-4.3546142129999993E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A92" s="3">
+        <v>33144</v>
+      </c>
+      <c r="B92" s="2">
+        <v>7.8855789519999997E-2</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A93" s="3">
+        <v>33238</v>
+      </c>
+      <c r="B93" s="2">
+        <v>1.1256070819999998E-2</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A94" s="3">
+        <v>33326</v>
+      </c>
+      <c r="B94" s="2">
+        <v>5.7849469940000002E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A95" s="3">
+        <v>33417</v>
+      </c>
+      <c r="B95" s="2">
+        <v>3.1944138269999998E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A96" s="3">
+        <v>33511</v>
+      </c>
+      <c r="B96" s="2">
+        <v>8.7439217429999994E-2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97" s="3">
+        <v>33603</v>
+      </c>
+      <c r="B97" s="2">
+        <v>-0.12352343960000001</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" s="3">
+        <v>33694</v>
+      </c>
+      <c r="B98" s="2">
+        <v>5.8668795090000003E-2</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" s="3">
+        <v>33785</v>
+      </c>
+      <c r="B99" s="2">
+        <v>5.18896811E-3</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" s="3">
+        <v>33877</v>
+      </c>
+      <c r="B100" s="2">
+        <v>0.10506126</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101" s="3">
+        <v>33969</v>
+      </c>
+      <c r="B101" s="2">
+        <v>-0.1172855439</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A102" s="3">
+        <v>34059</v>
+      </c>
+      <c r="B102" s="2">
+        <v>0.1189251487</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A103" s="3">
+        <v>34150</v>
+      </c>
+      <c r="B103" s="2">
+        <v>7.8917336099999999E-3</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A104" s="3">
+        <v>34242</v>
+      </c>
+      <c r="B104" s="2">
+        <v>-2.4907653039999998E-2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A105" s="3">
+        <v>34334</v>
+      </c>
+      <c r="B105" s="2">
+        <v>-9.2166580989999997E-2</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A106" s="3">
+        <v>34424</v>
+      </c>
+      <c r="B106" s="2">
+        <v>0.12403356880000001</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A107" s="3">
+        <v>34515</v>
+      </c>
+      <c r="B107" s="2">
+        <v>1.60092958E-2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A108" s="3">
+        <v>34607</v>
+      </c>
+      <c r="B108" s="2">
+        <v>4.2720231499999997E-2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A109" s="3">
+        <v>34698</v>
+      </c>
+      <c r="B109" s="2">
+        <v>-0.15379955880000001</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A110" s="3">
+        <v>34789</v>
+      </c>
+      <c r="B110" s="2">
+        <v>0.10382985259999999</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A111" s="3">
+        <v>34880</v>
+      </c>
+      <c r="B111" s="2">
+        <v>2.811719905E-2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112" s="3">
+        <v>34971</v>
+      </c>
+      <c r="B112" s="2">
+        <v>1.00936269E-2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A113" s="3">
+        <v>35062</v>
+      </c>
+      <c r="B113" s="2">
+        <v>-3.2818733519999997E-2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A114" s="3">
+        <v>35153</v>
+      </c>
+      <c r="B114" s="2">
+        <v>7.4807129559999991E-2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A115" s="3">
+        <v>35244</v>
+      </c>
+      <c r="B115" s="2">
+        <v>-3.4641529100000001E-3</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A116" s="3">
+        <v>35338</v>
+      </c>
+      <c r="B116" s="2">
+        <v>4.3584876099999996E-3</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A117" s="3">
+        <v>35430</v>
+      </c>
+      <c r="B117" s="2">
+        <v>-4.1763290010000002E-2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A118" s="3">
+        <v>35520</v>
+      </c>
+      <c r="B118" s="2">
+        <v>5.9276221800000001E-2</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A119" s="3">
+        <v>35611</v>
+      </c>
+      <c r="B119" s="2">
+        <v>-5.7106469000000005E-3</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A120" s="3">
+        <v>35703</v>
+      </c>
+      <c r="B120" s="2">
+        <v>1.012389006E-2</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A121" s="3">
+        <v>35795</v>
+      </c>
+      <c r="B121" s="2">
+        <v>-9.9581552030000006E-2</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A122" s="3">
+        <v>35885</v>
+      </c>
+      <c r="B122" s="2">
+        <v>0.10786337550000001</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A123" s="3">
+        <v>35976</v>
+      </c>
+      <c r="B123" s="2">
+        <v>-3.399749874E-2</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A124" s="3">
+        <v>36068</v>
+      </c>
+      <c r="B124" s="2">
+        <v>4.5000308199999998E-2</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A125" s="3">
+        <v>36160</v>
+      </c>
+      <c r="B125" s="2">
+        <v>-0.1927466089</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A126" s="3">
+        <v>36250</v>
+      </c>
+      <c r="B126" s="2">
+        <v>2.3743123769999999E-2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A127" s="3">
+        <v>36341</v>
+      </c>
+      <c r="B127" s="2">
+        <v>-8.7554136440000013E-2</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A128" s="3">
+        <v>36433</v>
+      </c>
+      <c r="B128" s="2">
+        <v>6.2469738799999994E-3</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A129" s="3">
+        <v>36525</v>
+      </c>
+      <c r="B129" s="2">
+        <v>-5.7362652020000002E-2</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A130" s="3">
+        <v>36616</v>
+      </c>
+      <c r="B130" s="2">
+        <v>5.5686101459999998E-2</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A131" s="3">
+        <v>36707</v>
+      </c>
+      <c r="B131" s="2">
+        <v>-1.8117313079999999E-2</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A132" s="3">
+        <v>36798</v>
+      </c>
+      <c r="B132" s="2">
+        <v>1.864290536E-2</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A133" s="3">
+        <v>36889</v>
+      </c>
+      <c r="B133" s="2">
+        <v>-2.5327264839999999E-2</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A134" s="3">
+        <v>36980</v>
+      </c>
+      <c r="B134" s="2">
+        <v>6.2251648540000003E-2</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A135" s="3">
+        <v>37071</v>
+      </c>
+      <c r="B135" s="2">
+        <v>4.0799684540000006E-2</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A136" s="3">
+        <v>37162</v>
+      </c>
+      <c r="B136" s="2">
+        <v>6.1135451370000003E-2</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A137" s="3">
+        <v>37256</v>
+      </c>
+      <c r="B137" s="2">
+        <v>-7.5305807089999996E-2</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A138" s="3">
+        <v>37344</v>
+      </c>
+      <c r="B138" s="2">
+        <v>4.9970852600000004E-2</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A139" s="3">
+        <v>37435</v>
+      </c>
+      <c r="B139" s="2">
+        <v>9.5988967799999995E-3</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A140" s="3">
+        <v>37529</v>
+      </c>
+      <c r="B140" s="2">
+        <v>2.673934457E-2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A141" s="3">
+        <v>37621</v>
+      </c>
+      <c r="B141" s="2">
+        <v>-0.10476379079999999</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A142" s="3">
+        <v>37711</v>
+      </c>
+      <c r="B142" s="2">
+        <v>5.23418535E-2</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A143" s="3">
+        <v>37802</v>
+      </c>
+      <c r="B143" s="2">
+        <v>2.5154011299999997E-2</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A144" s="3">
+        <v>37894</v>
+      </c>
+      <c r="B144" s="2">
+        <v>-4.268719176E-2</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A145" s="3">
+        <v>37986</v>
+      </c>
+      <c r="B145" s="2">
+        <v>-3.1972267540000002E-2</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A146" s="3">
+        <v>38077</v>
+      </c>
+      <c r="B146" s="2">
+        <v>0.1105157271</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A147" s="3">
+        <v>38168</v>
+      </c>
+      <c r="B147" s="2">
+        <v>1.273410921E-2</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A148" s="3">
+        <v>38260</v>
+      </c>
+      <c r="B148" s="2">
+        <v>4.8104654160000003E-2</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A149" s="3">
+        <v>38352</v>
+      </c>
+      <c r="B149" s="2">
+        <v>-5.1498419469999994E-2</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A150" s="3">
+        <v>38442</v>
+      </c>
+      <c r="B150" s="2">
+        <v>0.1016611197</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A151" s="3">
+        <v>38533</v>
+      </c>
+      <c r="B151" s="2">
+        <v>1.6481842360000002E-2</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A152" s="3">
+        <v>38625</v>
+      </c>
+      <c r="B152" s="2">
+        <v>2.8541620889999997E-2</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A153" s="3">
+        <v>38716</v>
+      </c>
+      <c r="B153" s="2">
+        <v>-9.1994223089999994E-2</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A154" s="3">
+        <v>38807</v>
+      </c>
+      <c r="B154" s="2">
+        <v>4.848397963E-2</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A155" s="3">
+        <v>38898</v>
+      </c>
+      <c r="B155" s="2">
+        <v>7.1263594600000004E-3</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A156" s="3">
+        <v>38989</v>
+      </c>
+      <c r="B156" s="2">
+        <v>5.1905026310000005E-2</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A157" s="3">
+        <v>39080</v>
+      </c>
+      <c r="B157" s="2">
+        <v>-2.907615819E-2</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A158" s="3">
+        <v>39171</v>
+      </c>
+      <c r="B158" s="2">
+        <v>9.1980129080000014E-2</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A159" s="3">
+        <v>39262</v>
+      </c>
+      <c r="B159" s="2">
+        <v>3.22793801E-3</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A160" s="3">
+        <v>39353</v>
+      </c>
+      <c r="B160" s="2">
+        <v>2.1503035659999999E-2</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A161" s="3">
+        <v>39447</v>
+      </c>
+      <c r="B161" s="2">
+        <v>-1.8347079700000001E-2</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A162" s="3">
+        <v>39538</v>
+      </c>
+      <c r="B162" s="2">
+        <v>0.10413868170000001</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A163" s="3">
+        <v>39629</v>
+      </c>
+      <c r="B163" s="2">
+        <v>-0.11671226230000001</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A164" s="3">
+        <v>39721</v>
+      </c>
+      <c r="B164" s="2">
+        <v>5.3337910369999998E-2</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A165" s="3">
+        <v>39813</v>
+      </c>
+      <c r="B165" s="2">
+        <v>-0.3007508794</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A166" s="3">
+        <v>39903</v>
+      </c>
+      <c r="B166" s="2">
+        <v>-5.392106428E-2</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A167" s="3">
+        <v>39994</v>
+      </c>
+      <c r="B167" s="2">
+        <v>-0.1537845464</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A168" s="3">
+        <v>40086</v>
+      </c>
+      <c r="B168" s="2">
+        <v>-1.5666474919999999E-2</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A169" s="3">
+        <v>40178</v>
+      </c>
+      <c r="B169" s="2">
+        <v>-0.1051725308</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A170" s="3">
+        <v>40268</v>
+      </c>
+      <c r="B170" s="2">
+        <v>8.0879804070000005E-2</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A171" s="3">
+        <v>40359</v>
+      </c>
+      <c r="B171" s="2">
+        <v>-2.7897510809999998E-2</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A172" s="3">
+        <v>40451</v>
+      </c>
+      <c r="B172" s="2">
+        <v>4.9490148699999998E-3</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A173" s="3">
+        <v>40543</v>
+      </c>
+      <c r="B173" s="2">
+        <v>-7.6121215909999998E-2</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A174" s="3">
+        <v>40633</v>
+      </c>
+      <c r="B174" s="2">
+        <v>5.3673323639999999E-2</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A175" s="3">
+        <v>40724</v>
+      </c>
+      <c r="B175" s="2">
+        <v>-3.0425955700000003E-3</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A176" s="3">
+        <v>40816</v>
+      </c>
+      <c r="B176" s="2">
+        <v>3.0332954499999999E-2</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A177" s="3">
+        <v>40907</v>
+      </c>
+      <c r="B177" s="2">
+        <v>-7.3738245999999995E-3</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A178" s="3">
+        <v>40998</v>
+      </c>
+      <c r="B178" s="2">
+        <v>2.2491355290000001E-2</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A179" s="3">
+        <v>41089</v>
+      </c>
+      <c r="B179" s="2">
+        <v>-6.2905316700000002E-3</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A180" s="3">
+        <v>41180</v>
+      </c>
+      <c r="B180" s="2">
+        <v>-3.10029938E-2</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A181" s="3">
+        <v>41274</v>
+      </c>
+      <c r="B181" s="2">
+        <v>-3.0925565169999999E-2</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A182" s="3">
+        <v>41362</v>
+      </c>
+      <c r="B182" s="2">
+        <v>-7.5767260099999997E-3</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A183" s="3">
+        <v>41453</v>
+      </c>
+      <c r="B183" s="2">
+        <v>-2.2957021000000001E-2</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A184" s="3"/>
+      <c r="B184" s="2"/>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A185" s="3"/>
+      <c r="B185" s="2"/>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A186" s="3"/>
+      <c r="B186" s="2"/>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A187" s="3"/>
+      <c r="B187" s="2"/>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A188" s="3"/>
+      <c r="B188" s="2"/>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A189" s="3"/>
+      <c r="B189" s="2"/>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A190" s="3"/>
+      <c r="B190" s="2"/>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A191" s="3"/>
+      <c r="B191" s="2"/>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A192" s="3"/>
+      <c r="B192" s="2"/>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A193" s="3"/>
+      <c r="B193" s="2"/>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A194" s="3"/>
+      <c r="B194" s="2"/>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A195" s="3"/>
+      <c r="B195" s="2"/>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A196" s="3"/>
+      <c r="B196" s="2"/>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A197" s="3"/>
+      <c r="B197" s="2"/>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A198" s="3"/>
+      <c r="B198" s="2"/>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A199" s="3"/>
+      <c r="B199" s="2"/>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A200" s="3"/>
+      <c r="B200" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>